<commit_message>
Add practice files for Deshpande Electricals & Motors onboarding
- Created 04-purchases.csv with a year of purchase records.
- Added 05-cost-list.csv detailing item costs and selling prices.
- Introduced 06-whatsapp-orders.txt containing WhatsApp order messages.
- Included 07-broken.xlsx as a test case for handling invalid files.
- Updated README.md to provide an overview of the practice pack and file usage.
- Added onboarding runbook in onboard-from-scratch.md for detailed setup instructions.
</commit_message>
<xml_diff>
--- a/demo/samples/bearings/03-outstanding.xlsx
+++ b/demo/samples/bearings/03-outstanding.xlsx
@@ -430,7 +430,7 @@
     <col width="28" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="14" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
+    <col width="22" customWidth="1" min="5" max="5"/>
     <col width="11" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
@@ -479,7 +479,7 @@
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Amount</t>
+          <t>Outstanding Amount</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">

</xml_diff>